<commit_message>
Update susunan bal Blok 10, 11, dan 12 (tambah dari atas) dan sinkronisasi laporan/web
</commit_message>
<xml_diff>
--- a/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
+++ b/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
@@ -29,6 +29,9 @@
     <sheet name="9 September" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="10 September" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="11 September" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="12 September" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="13 September" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="14 September" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -477,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H765"/>
+  <dimension ref="A1:H841"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -24594,6 +24597,2430 @@
         </is>
       </c>
       <c r="H765" s="2" t="inlineStr"/>
+    </row>
+    <row r="766" ht="20" customHeight="1">
+      <c r="A766" s="3" t="n">
+        <v>762</v>
+      </c>
+      <c r="B766" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C766" s="3" t="n">
+        <v>968</v>
+      </c>
+      <c r="D766" s="3" t="inlineStr">
+        <is>
+          <t>280139</t>
+        </is>
+      </c>
+      <c r="E766" s="3" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F766" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="G766" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H766" s="3" t="inlineStr"/>
+    </row>
+    <row r="767" ht="20" customHeight="1">
+      <c r="A767" s="2" t="n">
+        <v>763</v>
+      </c>
+      <c r="B767" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C767" s="2" t="n">
+        <v>969</v>
+      </c>
+      <c r="D767" s="2" t="inlineStr">
+        <is>
+          <t>280140</t>
+        </is>
+      </c>
+      <c r="E767" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="F767" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G767" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H767" s="2" t="inlineStr"/>
+    </row>
+    <row r="768" ht="20" customHeight="1">
+      <c r="A768" s="3" t="n">
+        <v>764</v>
+      </c>
+      <c r="B768" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C768" s="3" t="n">
+        <v>970</v>
+      </c>
+      <c r="D768" s="3" t="inlineStr">
+        <is>
+          <t>280141</t>
+        </is>
+      </c>
+      <c r="E768" s="3" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="F768" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="G768" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H768" s="3" t="inlineStr"/>
+    </row>
+    <row r="769" ht="20" customHeight="1">
+      <c r="A769" s="2" t="n">
+        <v>765</v>
+      </c>
+      <c r="B769" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C769" s="2" t="n">
+        <v>971</v>
+      </c>
+      <c r="D769" s="2" t="inlineStr">
+        <is>
+          <t>125987</t>
+        </is>
+      </c>
+      <c r="E769" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="F769" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="G769" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H769" s="2" t="inlineStr"/>
+    </row>
+    <row r="770" ht="20" customHeight="1">
+      <c r="A770" s="3" t="n">
+        <v>766</v>
+      </c>
+      <c r="B770" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C770" s="3" t="n">
+        <v>972</v>
+      </c>
+      <c r="D770" s="3" t="inlineStr">
+        <is>
+          <t>39841</t>
+        </is>
+      </c>
+      <c r="E770" s="3" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="F770" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="G770" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H770" s="3" t="inlineStr"/>
+    </row>
+    <row r="771" ht="20" customHeight="1">
+      <c r="A771" s="2" t="n">
+        <v>767</v>
+      </c>
+      <c r="B771" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C771" s="2" t="n">
+        <v>973</v>
+      </c>
+      <c r="D771" s="2" t="inlineStr">
+        <is>
+          <t>39842</t>
+        </is>
+      </c>
+      <c r="E771" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="F771" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="G771" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H771" s="2" t="inlineStr"/>
+    </row>
+    <row r="772" ht="20" customHeight="1">
+      <c r="A772" s="3" t="n">
+        <v>768</v>
+      </c>
+      <c r="B772" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C772" s="3" t="n">
+        <v>974</v>
+      </c>
+      <c r="D772" s="3" t="inlineStr"/>
+      <c r="E772" s="3" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="F772" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="G772" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H772" s="3" t="inlineStr"/>
+    </row>
+    <row r="773" ht="20" customHeight="1">
+      <c r="A773" s="2" t="n">
+        <v>769</v>
+      </c>
+      <c r="B773" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C773" s="2" t="n">
+        <v>975</v>
+      </c>
+      <c r="D773" s="2" t="inlineStr">
+        <is>
+          <t>280145</t>
+        </is>
+      </c>
+      <c r="E773" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F773" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="G773" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H773" s="2" t="inlineStr"/>
+    </row>
+    <row r="774" ht="20" customHeight="1">
+      <c r="A774" s="3" t="n">
+        <v>770</v>
+      </c>
+      <c r="B774" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C774" s="3" t="n">
+        <v>976</v>
+      </c>
+      <c r="D774" s="3" t="inlineStr">
+        <is>
+          <t>280146</t>
+        </is>
+      </c>
+      <c r="E774" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F774" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="G774" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H774" s="3" t="inlineStr"/>
+    </row>
+    <row r="775" ht="20" customHeight="1">
+      <c r="A775" s="2" t="n">
+        <v>771</v>
+      </c>
+      <c r="B775" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C775" s="2" t="n">
+        <v>977</v>
+      </c>
+      <c r="D775" s="2" t="inlineStr">
+        <is>
+          <t>280144</t>
+        </is>
+      </c>
+      <c r="E775" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F775" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G775" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H775" s="2" t="inlineStr"/>
+    </row>
+    <row r="776" ht="20" customHeight="1">
+      <c r="A776" s="3" t="n">
+        <v>772</v>
+      </c>
+      <c r="B776" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C776" s="3" t="n">
+        <v>978</v>
+      </c>
+      <c r="D776" s="3" t="inlineStr">
+        <is>
+          <t>125822</t>
+        </is>
+      </c>
+      <c r="E776" s="3" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="F776" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="G776" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H776" s="3" t="inlineStr"/>
+    </row>
+    <row r="777" ht="20" customHeight="1">
+      <c r="A777" s="2" t="n">
+        <v>773</v>
+      </c>
+      <c r="B777" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C777" s="2" t="n">
+        <v>979</v>
+      </c>
+      <c r="D777" s="2" t="inlineStr">
+        <is>
+          <t>125821</t>
+        </is>
+      </c>
+      <c r="E777" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="F777" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G777" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H777" s="2" t="inlineStr"/>
+    </row>
+    <row r="778" ht="20" customHeight="1">
+      <c r="A778" s="3" t="n">
+        <v>774</v>
+      </c>
+      <c r="B778" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C778" s="3" t="n">
+        <v>980</v>
+      </c>
+      <c r="D778" s="3" t="inlineStr">
+        <is>
+          <t>280302</t>
+        </is>
+      </c>
+      <c r="E778" s="3" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="F778" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="G778" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H778" s="3" t="inlineStr"/>
+    </row>
+    <row r="779" ht="20" customHeight="1">
+      <c r="A779" s="2" t="n">
+        <v>775</v>
+      </c>
+      <c r="B779" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C779" s="2" t="n">
+        <v>981</v>
+      </c>
+      <c r="D779" s="2" t="inlineStr">
+        <is>
+          <t>125991</t>
+        </is>
+      </c>
+      <c r="E779" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="F779" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G779" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H779" s="2" t="inlineStr"/>
+    </row>
+    <row r="780" ht="20" customHeight="1">
+      <c r="A780" s="3" t="n">
+        <v>776</v>
+      </c>
+      <c r="B780" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C780" s="3" t="n">
+        <v>982</v>
+      </c>
+      <c r="D780" s="3" t="inlineStr">
+        <is>
+          <t>125990</t>
+        </is>
+      </c>
+      <c r="E780" s="3" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="F780" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="G780" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H780" s="3" t="inlineStr"/>
+    </row>
+    <row r="781" ht="20" customHeight="1">
+      <c r="A781" s="2" t="n">
+        <v>777</v>
+      </c>
+      <c r="B781" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C781" s="2" t="n">
+        <v>983</v>
+      </c>
+      <c r="D781" s="2" t="inlineStr">
+        <is>
+          <t>125992</t>
+        </is>
+      </c>
+      <c r="E781" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="F781" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="G781" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H781" s="2" t="inlineStr"/>
+    </row>
+    <row r="782" ht="20" customHeight="1">
+      <c r="A782" s="3" t="n">
+        <v>778</v>
+      </c>
+      <c r="B782" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C782" s="3" t="n">
+        <v>984</v>
+      </c>
+      <c r="D782" s="3" t="inlineStr">
+        <is>
+          <t>125988</t>
+        </is>
+      </c>
+      <c r="E782" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F782" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="G782" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H782" s="3" t="inlineStr"/>
+    </row>
+    <row r="783" ht="20" customHeight="1">
+      <c r="A783" s="2" t="n">
+        <v>779</v>
+      </c>
+      <c r="B783" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C783" s="2" t="n">
+        <v>985</v>
+      </c>
+      <c r="D783" s="2" t="inlineStr">
+        <is>
+          <t>280143</t>
+        </is>
+      </c>
+      <c r="E783" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F783" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G783" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H783" s="2" t="inlineStr"/>
+    </row>
+    <row r="784" ht="20" customHeight="1">
+      <c r="A784" s="3" t="n">
+        <v>780</v>
+      </c>
+      <c r="B784" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C784" s="3" t="n">
+        <v>986</v>
+      </c>
+      <c r="D784" s="3" t="inlineStr">
+        <is>
+          <t>125989</t>
+        </is>
+      </c>
+      <c r="E784" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F784" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="G784" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H784" s="3" t="inlineStr"/>
+    </row>
+    <row r="785" ht="20" customHeight="1">
+      <c r="A785" s="2" t="n">
+        <v>781</v>
+      </c>
+      <c r="B785" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C785" s="2" t="n">
+        <v>987</v>
+      </c>
+      <c r="D785" s="2" t="inlineStr">
+        <is>
+          <t>280142</t>
+        </is>
+      </c>
+      <c r="E785" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F785" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="G785" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H785" s="2" t="inlineStr"/>
+    </row>
+    <row r="786" ht="20" customHeight="1">
+      <c r="A786" s="3" t="n">
+        <v>782</v>
+      </c>
+      <c r="B786" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C786" s="3" t="n">
+        <v>991</v>
+      </c>
+      <c r="D786" s="3" t="inlineStr">
+        <is>
+          <t>280619</t>
+        </is>
+      </c>
+      <c r="E786" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F786" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="G786" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H786" s="3" t="inlineStr"/>
+    </row>
+    <row r="787" ht="20" customHeight="1">
+      <c r="A787" s="2" t="n">
+        <v>783</v>
+      </c>
+      <c r="B787" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C787" s="2" t="n">
+        <v>992</v>
+      </c>
+      <c r="D787" s="2" t="inlineStr">
+        <is>
+          <t>280763</t>
+        </is>
+      </c>
+      <c r="E787" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F787" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="G787" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H787" s="2" t="inlineStr"/>
+    </row>
+    <row r="788" ht="20" customHeight="1">
+      <c r="A788" s="3" t="n">
+        <v>784</v>
+      </c>
+      <c r="B788" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C788" s="3" t="n">
+        <v>993</v>
+      </c>
+      <c r="D788" s="3" t="inlineStr">
+        <is>
+          <t>280618</t>
+        </is>
+      </c>
+      <c r="E788" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F788" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="G788" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H788" s="3" t="inlineStr"/>
+    </row>
+    <row r="789" ht="20" customHeight="1">
+      <c r="A789" s="2" t="n">
+        <v>785</v>
+      </c>
+      <c r="B789" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C789" s="2" t="n">
+        <v>994</v>
+      </c>
+      <c r="D789" s="2" t="inlineStr">
+        <is>
+          <t>280762</t>
+        </is>
+      </c>
+      <c r="E789" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F789" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="G789" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H789" s="2" t="inlineStr"/>
+    </row>
+    <row r="790" ht="20" customHeight="1">
+      <c r="A790" s="3" t="n">
+        <v>786</v>
+      </c>
+      <c r="B790" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C790" s="3" t="n">
+        <v>995</v>
+      </c>
+      <c r="D790" s="3" t="inlineStr">
+        <is>
+          <t>39844</t>
+        </is>
+      </c>
+      <c r="E790" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="F790" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="G790" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H790" s="3" t="inlineStr"/>
+    </row>
+    <row r="791" ht="20" customHeight="1">
+      <c r="A791" s="2" t="n">
+        <v>787</v>
+      </c>
+      <c r="B791" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C791" s="2" t="n">
+        <v>996</v>
+      </c>
+      <c r="D791" s="2" t="inlineStr">
+        <is>
+          <t>39843</t>
+        </is>
+      </c>
+      <c r="E791" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="F791" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="G791" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H791" s="2" t="inlineStr"/>
+    </row>
+    <row r="792" ht="20" customHeight="1">
+      <c r="A792" s="3" t="n">
+        <v>788</v>
+      </c>
+      <c r="B792" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C792" s="3" t="n">
+        <v>997</v>
+      </c>
+      <c r="D792" s="3" t="inlineStr">
+        <is>
+          <t>280617</t>
+        </is>
+      </c>
+      <c r="E792" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F792" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="G792" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H792" s="3" t="inlineStr"/>
+    </row>
+    <row r="793" ht="20" customHeight="1">
+      <c r="A793" s="2" t="n">
+        <v>789</v>
+      </c>
+      <c r="B793" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C793" s="2" t="n">
+        <v>998</v>
+      </c>
+      <c r="D793" s="2" t="inlineStr">
+        <is>
+          <t>280761</t>
+        </is>
+      </c>
+      <c r="E793" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F793" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G793" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H793" s="2" t="inlineStr"/>
+    </row>
+    <row r="794" ht="20" customHeight="1">
+      <c r="A794" s="3" t="n">
+        <v>790</v>
+      </c>
+      <c r="B794" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C794" s="3" t="n">
+        <v>999</v>
+      </c>
+      <c r="D794" s="3" t="inlineStr">
+        <is>
+          <t>280616</t>
+        </is>
+      </c>
+      <c r="E794" s="3" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="F794" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="G794" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H794" s="3" t="inlineStr"/>
+    </row>
+    <row r="795" ht="20" customHeight="1">
+      <c r="A795" s="2" t="n">
+        <v>791</v>
+      </c>
+      <c r="B795" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C795" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D795" s="2" t="inlineStr">
+        <is>
+          <t>125833</t>
+        </is>
+      </c>
+      <c r="E795" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="F795" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G795" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H795" s="2" t="inlineStr"/>
+    </row>
+    <row r="796" ht="20" customHeight="1">
+      <c r="A796" s="3" t="n">
+        <v>792</v>
+      </c>
+      <c r="B796" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C796" s="3" t="n">
+        <v>1001</v>
+      </c>
+      <c r="D796" s="3" t="inlineStr">
+        <is>
+          <t>280613</t>
+        </is>
+      </c>
+      <c r="E796" s="3" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="F796" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="G796" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H796" s="3" t="inlineStr"/>
+    </row>
+    <row r="797" ht="20" customHeight="1">
+      <c r="A797" s="2" t="n">
+        <v>793</v>
+      </c>
+      <c r="B797" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C797" s="2" t="n">
+        <v>1002</v>
+      </c>
+      <c r="D797" s="2" t="inlineStr"/>
+      <c r="E797" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="F797" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="G797" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H797" s="2" t="inlineStr"/>
+    </row>
+    <row r="798" ht="20" customHeight="1">
+      <c r="A798" s="3" t="n">
+        <v>794</v>
+      </c>
+      <c r="B798" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C798" s="3" t="n">
+        <v>1003</v>
+      </c>
+      <c r="D798" s="3" t="inlineStr">
+        <is>
+          <t>125832</t>
+        </is>
+      </c>
+      <c r="E798" s="3" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="F798" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="G798" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H798" s="3" t="inlineStr"/>
+    </row>
+    <row r="799" ht="20" customHeight="1">
+      <c r="A799" s="2" t="n">
+        <v>795</v>
+      </c>
+      <c r="B799" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C799" s="2" t="n">
+        <v>1004</v>
+      </c>
+      <c r="D799" s="2" t="inlineStr">
+        <is>
+          <t>125862</t>
+        </is>
+      </c>
+      <c r="E799" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F799" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="G799" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H799" s="2" t="inlineStr"/>
+    </row>
+    <row r="800" ht="20" customHeight="1">
+      <c r="A800" s="3" t="n">
+        <v>796</v>
+      </c>
+      <c r="B800" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C800" s="3" t="n">
+        <v>1005</v>
+      </c>
+      <c r="D800" s="3" t="inlineStr">
+        <is>
+          <t>125866</t>
+        </is>
+      </c>
+      <c r="E800" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F800" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="G800" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H800" s="3" t="inlineStr"/>
+    </row>
+    <row r="801" ht="20" customHeight="1">
+      <c r="A801" s="2" t="n">
+        <v>797</v>
+      </c>
+      <c r="B801" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C801" s="2" t="n">
+        <v>1006</v>
+      </c>
+      <c r="D801" s="2" t="inlineStr">
+        <is>
+          <t>125863</t>
+        </is>
+      </c>
+      <c r="E801" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F801" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G801" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H801" s="2" t="inlineStr"/>
+    </row>
+    <row r="802" ht="20" customHeight="1">
+      <c r="A802" s="3" t="n">
+        <v>798</v>
+      </c>
+      <c r="B802" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C802" s="3" t="n">
+        <v>1007</v>
+      </c>
+      <c r="D802" s="3" t="inlineStr">
+        <is>
+          <t>125864</t>
+        </is>
+      </c>
+      <c r="E802" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F802" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="G802" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H802" s="3" t="inlineStr"/>
+    </row>
+    <row r="803" ht="20" customHeight="1">
+      <c r="A803" s="2" t="n">
+        <v>799</v>
+      </c>
+      <c r="B803" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C803" s="2" t="n">
+        <v>1008</v>
+      </c>
+      <c r="D803" s="2" t="inlineStr">
+        <is>
+          <t>125865</t>
+        </is>
+      </c>
+      <c r="E803" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F803" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="G803" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H803" s="2" t="inlineStr"/>
+    </row>
+    <row r="804" ht="20" customHeight="1">
+      <c r="A804" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="B804" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C804" s="3" t="n">
+        <v>1009</v>
+      </c>
+      <c r="D804" s="3" t="inlineStr">
+        <is>
+          <t>125831</t>
+        </is>
+      </c>
+      <c r="E804" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F804" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="G804" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H804" s="3" t="inlineStr"/>
+    </row>
+    <row r="805" ht="20" customHeight="1">
+      <c r="A805" s="2" t="n">
+        <v>801</v>
+      </c>
+      <c r="B805" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C805" s="2" t="n">
+        <v>1010</v>
+      </c>
+      <c r="D805" s="2" t="inlineStr">
+        <is>
+          <t>280760</t>
+        </is>
+      </c>
+      <c r="E805" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F805" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="G805" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H805" s="2" t="inlineStr"/>
+    </row>
+    <row r="806" ht="20" customHeight="1">
+      <c r="A806" s="3" t="n">
+        <v>802</v>
+      </c>
+      <c r="B806" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C806" s="3" t="n">
+        <v>1011</v>
+      </c>
+      <c r="D806" s="3" t="inlineStr">
+        <is>
+          <t>280614</t>
+        </is>
+      </c>
+      <c r="E806" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F806" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="G806" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H806" s="3" t="inlineStr"/>
+    </row>
+    <row r="807" ht="20" customHeight="1">
+      <c r="A807" s="2" t="n">
+        <v>803</v>
+      </c>
+      <c r="B807" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C807" s="2" t="n">
+        <v>1012</v>
+      </c>
+      <c r="D807" s="2" t="inlineStr">
+        <is>
+          <t>280612</t>
+        </is>
+      </c>
+      <c r="E807" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F807" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="G807" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H807" s="2" t="inlineStr"/>
+    </row>
+    <row r="808" ht="20" customHeight="1">
+      <c r="A808" s="3" t="n">
+        <v>804</v>
+      </c>
+      <c r="B808" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C808" s="3" t="n">
+        <v>1013</v>
+      </c>
+      <c r="D808" s="3" t="inlineStr">
+        <is>
+          <t>280759</t>
+        </is>
+      </c>
+      <c r="E808" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F808" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="G808" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H808" s="3" t="inlineStr"/>
+    </row>
+    <row r="809" ht="20" customHeight="1">
+      <c r="A809" s="2" t="n">
+        <v>805</v>
+      </c>
+      <c r="B809" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C809" s="2" t="n">
+        <v>1014</v>
+      </c>
+      <c r="D809" s="2" t="inlineStr">
+        <is>
+          <t>280615</t>
+        </is>
+      </c>
+      <c r="E809" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F809" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="G809" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H809" s="2" t="inlineStr"/>
+    </row>
+    <row r="810" ht="20" customHeight="1">
+      <c r="A810" s="3" t="n">
+        <v>806</v>
+      </c>
+      <c r="B810" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C810" s="3" t="n">
+        <v>1015</v>
+      </c>
+      <c r="D810" s="3" t="inlineStr">
+        <is>
+          <t>280620</t>
+        </is>
+      </c>
+      <c r="E810" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F810" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="G810" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H810" s="3" t="inlineStr"/>
+    </row>
+    <row r="811" ht="20" customHeight="1">
+      <c r="A811" s="2" t="n">
+        <v>807</v>
+      </c>
+      <c r="B811" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C811" s="2" t="n">
+        <v>1016</v>
+      </c>
+      <c r="D811" s="2" t="inlineStr">
+        <is>
+          <t>280611</t>
+        </is>
+      </c>
+      <c r="E811" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="F811" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="G811" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H811" s="2" t="inlineStr"/>
+    </row>
+    <row r="812" ht="20" customHeight="1">
+      <c r="A812" s="3" t="n">
+        <v>808</v>
+      </c>
+      <c r="B812" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C812" s="3" t="n">
+        <v>1017</v>
+      </c>
+      <c r="D812" s="3" t="inlineStr">
+        <is>
+          <t>280412</t>
+        </is>
+      </c>
+      <c r="E812" s="3" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="F812" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="G812" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H812" s="3" t="inlineStr"/>
+    </row>
+    <row r="813" ht="20" customHeight="1">
+      <c r="A813" s="2" t="n">
+        <v>809</v>
+      </c>
+      <c r="B813" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C813" s="2" t="n">
+        <v>1018</v>
+      </c>
+      <c r="D813" s="2" t="inlineStr">
+        <is>
+          <t>280299</t>
+        </is>
+      </c>
+      <c r="E813" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F813" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="G813" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H813" s="2" t="inlineStr"/>
+    </row>
+    <row r="814" ht="20" customHeight="1">
+      <c r="A814" s="3" t="n">
+        <v>810</v>
+      </c>
+      <c r="B814" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C814" s="3" t="n">
+        <v>1019</v>
+      </c>
+      <c r="D814" s="3" t="inlineStr">
+        <is>
+          <t>280300</t>
+        </is>
+      </c>
+      <c r="E814" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F814" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="G814" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H814" s="3" t="inlineStr"/>
+    </row>
+    <row r="815" ht="20" customHeight="1">
+      <c r="A815" s="2" t="n">
+        <v>811</v>
+      </c>
+      <c r="B815" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C815" s="2" t="n">
+        <v>1020</v>
+      </c>
+      <c r="D815" s="2" t="inlineStr">
+        <is>
+          <t>282168</t>
+        </is>
+      </c>
+      <c r="E815" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F815" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="G815" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H815" s="2" t="inlineStr"/>
+    </row>
+    <row r="816" ht="20" customHeight="1">
+      <c r="A816" s="3" t="n">
+        <v>812</v>
+      </c>
+      <c r="B816" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C816" s="3" t="n">
+        <v>1021</v>
+      </c>
+      <c r="D816" s="3" t="inlineStr">
+        <is>
+          <t>282096</t>
+        </is>
+      </c>
+      <c r="E816" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F816" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="G816" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H816" s="3" t="inlineStr"/>
+    </row>
+    <row r="817" ht="20" customHeight="1">
+      <c r="A817" s="2" t="n">
+        <v>813</v>
+      </c>
+      <c r="B817" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C817" s="2" t="n">
+        <v>1022</v>
+      </c>
+      <c r="D817" s="2" t="inlineStr">
+        <is>
+          <t>282097</t>
+        </is>
+      </c>
+      <c r="E817" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F817" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G817" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H817" s="2" t="inlineStr"/>
+    </row>
+    <row r="818" ht="20" customHeight="1">
+      <c r="A818" s="3" t="n">
+        <v>814</v>
+      </c>
+      <c r="B818" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C818" s="3" t="n">
+        <v>1023</v>
+      </c>
+      <c r="D818" s="3" t="inlineStr">
+        <is>
+          <t>282098</t>
+        </is>
+      </c>
+      <c r="E818" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F818" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="G818" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H818" s="3" t="inlineStr"/>
+    </row>
+    <row r="819" ht="20" customHeight="1">
+      <c r="A819" s="2" t="n">
+        <v>815</v>
+      </c>
+      <c r="B819" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C819" s="2" t="n">
+        <v>1024</v>
+      </c>
+      <c r="D819" s="2" t="inlineStr">
+        <is>
+          <t>282171</t>
+        </is>
+      </c>
+      <c r="E819" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F819" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G819" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H819" s="2" t="inlineStr"/>
+    </row>
+    <row r="820" ht="20" customHeight="1">
+      <c r="A820" s="3" t="n">
+        <v>816</v>
+      </c>
+      <c r="B820" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C820" s="3" t="n">
+        <v>1025</v>
+      </c>
+      <c r="D820" s="3" t="inlineStr">
+        <is>
+          <t>282174</t>
+        </is>
+      </c>
+      <c r="E820" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F820" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="G820" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H820" s="3" t="inlineStr"/>
+    </row>
+    <row r="821" ht="20" customHeight="1">
+      <c r="A821" s="2" t="n">
+        <v>817</v>
+      </c>
+      <c r="B821" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C821" s="2" t="n">
+        <v>1026</v>
+      </c>
+      <c r="D821" s="2" t="inlineStr">
+        <is>
+          <t>282173</t>
+        </is>
+      </c>
+      <c r="E821" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F821" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="G821" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H821" s="2" t="inlineStr"/>
+    </row>
+    <row r="822" ht="20" customHeight="1">
+      <c r="A822" s="3" t="n">
+        <v>818</v>
+      </c>
+      <c r="B822" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C822" s="3" t="n">
+        <v>1027</v>
+      </c>
+      <c r="D822" s="3" t="inlineStr">
+        <is>
+          <t>282176</t>
+        </is>
+      </c>
+      <c r="E822" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F822" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="G822" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H822" s="3" t="inlineStr"/>
+    </row>
+    <row r="823" ht="20" customHeight="1">
+      <c r="A823" s="2" t="n">
+        <v>819</v>
+      </c>
+      <c r="B823" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C823" s="2" t="n">
+        <v>1028</v>
+      </c>
+      <c r="D823" s="2" t="inlineStr">
+        <is>
+          <t>282169</t>
+        </is>
+      </c>
+      <c r="E823" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F823" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G823" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H823" s="2" t="inlineStr"/>
+    </row>
+    <row r="824" ht="20" customHeight="1">
+      <c r="A824" s="3" t="n">
+        <v>820</v>
+      </c>
+      <c r="B824" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C824" s="3" t="n">
+        <v>1029</v>
+      </c>
+      <c r="D824" s="3" t="inlineStr">
+        <is>
+          <t>282170</t>
+        </is>
+      </c>
+      <c r="E824" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F824" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="G824" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H824" s="3" t="inlineStr"/>
+    </row>
+    <row r="825" ht="20" customHeight="1">
+      <c r="A825" s="2" t="n">
+        <v>821</v>
+      </c>
+      <c r="B825" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C825" s="2" t="n">
+        <v>1030</v>
+      </c>
+      <c r="D825" s="2" t="inlineStr">
+        <is>
+          <t>282175</t>
+        </is>
+      </c>
+      <c r="E825" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F825" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="G825" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H825" s="2" t="inlineStr"/>
+    </row>
+    <row r="826" ht="20" customHeight="1">
+      <c r="A826" s="3" t="n">
+        <v>822</v>
+      </c>
+      <c r="B826" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C826" s="3" t="n">
+        <v>1031</v>
+      </c>
+      <c r="D826" s="3" t="inlineStr">
+        <is>
+          <t>282252</t>
+        </is>
+      </c>
+      <c r="E826" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F826" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="G826" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H826" s="3" t="inlineStr"/>
+    </row>
+    <row r="827" ht="20" customHeight="1">
+      <c r="A827" s="2" t="n">
+        <v>823</v>
+      </c>
+      <c r="B827" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C827" s="2" t="n">
+        <v>1032</v>
+      </c>
+      <c r="D827" s="2" t="inlineStr">
+        <is>
+          <t>282228</t>
+        </is>
+      </c>
+      <c r="E827" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F827" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G827" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H827" s="2" t="inlineStr"/>
+    </row>
+    <row r="828" ht="20" customHeight="1">
+      <c r="A828" s="3" t="n">
+        <v>824</v>
+      </c>
+      <c r="B828" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C828" s="3" t="n">
+        <v>1033</v>
+      </c>
+      <c r="D828" s="3" t="inlineStr">
+        <is>
+          <t>282099</t>
+        </is>
+      </c>
+      <c r="E828" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F828" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="G828" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H828" s="3" t="inlineStr"/>
+    </row>
+    <row r="829" ht="20" customHeight="1">
+      <c r="A829" s="2" t="n">
+        <v>825</v>
+      </c>
+      <c r="B829" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C829" s="2" t="n">
+        <v>1034</v>
+      </c>
+      <c r="D829" s="2" t="inlineStr">
+        <is>
+          <t>282251</t>
+        </is>
+      </c>
+      <c r="E829" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F829" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="G829" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H829" s="2" t="inlineStr"/>
+    </row>
+    <row r="830" ht="20" customHeight="1">
+      <c r="A830" s="3" t="n">
+        <v>826</v>
+      </c>
+      <c r="B830" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C830" s="3" t="n">
+        <v>1035</v>
+      </c>
+      <c r="D830" s="3" t="inlineStr">
+        <is>
+          <t>282100</t>
+        </is>
+      </c>
+      <c r="E830" s="3" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F830" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="G830" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H830" s="3" t="inlineStr"/>
+    </row>
+    <row r="831" ht="20" customHeight="1">
+      <c r="A831" s="2" t="n">
+        <v>827</v>
+      </c>
+      <c r="B831" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C831" s="2" t="n">
+        <v>1036</v>
+      </c>
+      <c r="D831" s="2" t="inlineStr">
+        <is>
+          <t>280315</t>
+        </is>
+      </c>
+      <c r="E831" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F831" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="G831" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H831" s="2" t="inlineStr"/>
+    </row>
+    <row r="832" ht="20" customHeight="1">
+      <c r="A832" s="3" t="n">
+        <v>828</v>
+      </c>
+      <c r="B832" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C832" s="3" t="n">
+        <v>1037</v>
+      </c>
+      <c r="D832" s="3" t="inlineStr">
+        <is>
+          <t>280314</t>
+        </is>
+      </c>
+      <c r="E832" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F832" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="G832" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H832" s="3" t="inlineStr"/>
+    </row>
+    <row r="833" ht="20" customHeight="1">
+      <c r="A833" s="2" t="n">
+        <v>829</v>
+      </c>
+      <c r="B833" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C833" s="2" t="n">
+        <v>1038</v>
+      </c>
+      <c r="D833" s="2" t="inlineStr">
+        <is>
+          <t>282172</t>
+        </is>
+      </c>
+      <c r="E833" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F833" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="G833" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H833" s="2" t="inlineStr"/>
+    </row>
+    <row r="834" ht="20" customHeight="1">
+      <c r="A834" s="3" t="n">
+        <v>830</v>
+      </c>
+      <c r="B834" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C834" s="3" t="n">
+        <v>1039</v>
+      </c>
+      <c r="D834" s="3" t="inlineStr">
+        <is>
+          <t>282229</t>
+        </is>
+      </c>
+      <c r="E834" s="3" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="F834" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="G834" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H834" s="3" t="inlineStr"/>
+    </row>
+    <row r="835" ht="20" customHeight="1">
+      <c r="A835" s="2" t="n">
+        <v>831</v>
+      </c>
+      <c r="B835" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C835" s="2" t="n">
+        <v>1040</v>
+      </c>
+      <c r="D835" s="2" t="inlineStr">
+        <is>
+          <t>282253</t>
+        </is>
+      </c>
+      <c r="E835" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="F835" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="G835" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H835" s="2" t="inlineStr"/>
+    </row>
+    <row r="836" ht="20" customHeight="1">
+      <c r="A836" s="3" t="n">
+        <v>832</v>
+      </c>
+      <c r="B836" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C836" s="3" t="n">
+        <v>1041</v>
+      </c>
+      <c r="D836" s="3" t="inlineStr">
+        <is>
+          <t>282230</t>
+        </is>
+      </c>
+      <c r="E836" s="3" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F836" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="G836" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H836" s="3" t="inlineStr"/>
+    </row>
+    <row r="837" ht="20" customHeight="1">
+      <c r="A837" s="2" t="n">
+        <v>833</v>
+      </c>
+      <c r="B837" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C837" s="2" t="n">
+        <v>1042</v>
+      </c>
+      <c r="D837" s="2" t="inlineStr">
+        <is>
+          <t>282231</t>
+        </is>
+      </c>
+      <c r="E837" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F837" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G837" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H837" s="2" t="inlineStr"/>
+    </row>
+    <row r="838" ht="20" customHeight="1">
+      <c r="A838" s="3" t="n">
+        <v>834</v>
+      </c>
+      <c r="B838" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C838" s="3" t="n">
+        <v>1043</v>
+      </c>
+      <c r="D838" s="3" t="inlineStr">
+        <is>
+          <t>282167</t>
+        </is>
+      </c>
+      <c r="E838" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F838" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="G838" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H838" s="3" t="inlineStr"/>
+    </row>
+    <row r="839" ht="20" customHeight="1">
+      <c r="A839" s="2" t="n">
+        <v>835</v>
+      </c>
+      <c r="B839" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C839" s="2" t="n">
+        <v>1044</v>
+      </c>
+      <c r="D839" s="2" t="inlineStr">
+        <is>
+          <t>282166</t>
+        </is>
+      </c>
+      <c r="E839" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F839" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="G839" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H839" s="2" t="inlineStr"/>
+    </row>
+    <row r="840" ht="20" customHeight="1">
+      <c r="A840" s="3" t="n">
+        <v>836</v>
+      </c>
+      <c r="B840" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C840" s="3" t="n">
+        <v>1045</v>
+      </c>
+      <c r="D840" s="3" t="inlineStr">
+        <is>
+          <t>282416</t>
+        </is>
+      </c>
+      <c r="E840" s="3" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F840" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="G840" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H840" s="3" t="inlineStr"/>
+    </row>
+    <row r="841" ht="20" customHeight="1">
+      <c r="A841" s="2" t="n">
+        <v>837</v>
+      </c>
+      <c r="B841" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C841" s="2" t="n">
+        <v>1046</v>
+      </c>
+      <c r="D841" s="2" t="inlineStr">
+        <is>
+          <t>282095</t>
+        </is>
+      </c>
+      <c r="E841" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F841" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="G841" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H841" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -37002,6 +39429,2239 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>No Gudang</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Nomor Barcode</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Berat (Kg)</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>968</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>280139</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>969</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>280140</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>970</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>280141</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>971</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>125987</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>972</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>39841</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>973</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>39842</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>974</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>975</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>280145</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>976</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>280146</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>977</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>280144</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>978</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>125822</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>979</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>125821</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>980</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>280302</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>981</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>125991</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>982</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>125990</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>983</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>125992</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>984</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>125988</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>985</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>280143</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>986</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>125989</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>987</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>280142</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>No Gudang</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Nomor Barcode</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Berat (Kg)</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>991</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>280619</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>992</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>280763</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>993</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>280618</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>994</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>280762</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>995</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>39844</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>996</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>39843</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>997</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>280617</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>998</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>280761</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>999</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>280616</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>125833</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>1001</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>280613</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>1002</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>1003</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>125832</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>1004</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>125862</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>1005</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>125866</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1006</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>125863</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>1007</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>125864</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>1008</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>125865</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>1009</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>125831</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>1010</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>280760</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>1011</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>280614</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>1012</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>280612</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>1013</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>280759</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>1014</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>280615</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>1015</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>280620</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>1016</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>280611</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>1017</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>280412</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>1018</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>280299</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>1019</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>280300</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>No Gudang</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Nomor Barcode</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Berat (Kg)</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>1020</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>282168</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1021</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>282096</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>1022</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>282097</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>1023</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>282098</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>1024</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>282171</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>1025</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>282174</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>1026</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>282173</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>1027</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>282176</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>1028</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>282169</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>1029</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>282170</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>1030</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>282175</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>1031</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>282252</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>1032</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>282228</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>1033</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>282099</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>1034</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>282251</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1035</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>282100</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>1036</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>280315</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>1037</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>280314</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>1038</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>282172</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>1039</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>282229</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>1040</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>282253</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>1041</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>282230</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>1042</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>282231</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>1043</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>282167</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>1044</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>282166</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>1045</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>282416</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>1046</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>282095</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat: sinkronisasi Cek Barkot Supabase dengan pagination dan regenerasi laporan
</commit_message>
<xml_diff>
--- a/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
+++ b/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
@@ -35,6 +35,7 @@
     <sheet name="17 September" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="18 September" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="19 September" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="20 September" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -483,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H959"/>
+  <dimension ref="A1:H975"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -30295,24 +30296,24 @@
       </c>
       <c r="B944" s="3" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="C944" s="3" t="n">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="D944" s="3" t="inlineStr">
         <is>
-          <t>286375</t>
+          <t>374136</t>
         </is>
       </c>
       <c r="E944" s="3" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>65</t>
         </is>
       </c>
       <c r="F944" s="3" t="n">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="G944" s="3" t="inlineStr">
         <is>
@@ -30331,20 +30332,20 @@
         </is>
       </c>
       <c r="C945" s="2" t="n">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="D945" s="2" t="inlineStr">
         <is>
-          <t>286373</t>
+          <t>286375</t>
         </is>
       </c>
       <c r="E945" s="2" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>72</t>
         </is>
       </c>
       <c r="F945" s="2" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G945" s="2" t="inlineStr">
         <is>
@@ -30363,20 +30364,20 @@
         </is>
       </c>
       <c r="C946" s="3" t="n">
-        <v>1190</v>
+        <v>1186</v>
       </c>
       <c r="D946" s="3" t="inlineStr">
         <is>
-          <t>286057</t>
+          <t>286373</t>
         </is>
       </c>
       <c r="E946" s="3" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>74</t>
         </is>
       </c>
       <c r="F946" s="3" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G946" s="3" t="inlineStr">
         <is>
@@ -30391,15 +30392,15 @@
       </c>
       <c r="B947" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="C947" s="2" t="n">
-        <v>1191</v>
+        <v>1189</v>
       </c>
       <c r="D947" s="2" t="inlineStr">
         <is>
-          <t>282939</t>
+          <t>374140</t>
         </is>
       </c>
       <c r="E947" s="2" t="inlineStr">
@@ -30408,7 +30409,7 @@
         </is>
       </c>
       <c r="F947" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="G947" s="2" t="inlineStr">
         <is>
@@ -30427,20 +30428,20 @@
         </is>
       </c>
       <c r="C948" s="3" t="n">
-        <v>1194</v>
+        <v>1190</v>
       </c>
       <c r="D948" s="3" t="inlineStr">
         <is>
-          <t>284796</t>
+          <t>286057</t>
         </is>
       </c>
       <c r="E948" s="3" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>68</t>
         </is>
       </c>
       <c r="F948" s="3" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G948" s="3" t="inlineStr">
         <is>
@@ -30459,20 +30460,20 @@
         </is>
       </c>
       <c r="C949" s="2" t="n">
-        <v>1196</v>
+        <v>1191</v>
       </c>
       <c r="D949" s="2" t="inlineStr">
         <is>
-          <t>286370</t>
+          <t>282939</t>
         </is>
       </c>
       <c r="E949" s="2" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>65</t>
         </is>
       </c>
       <c r="F949" s="2" t="n">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="G949" s="2" t="inlineStr">
         <is>
@@ -30487,24 +30488,24 @@
       </c>
       <c r="B950" s="3" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="C950" s="3" t="n">
-        <v>1198</v>
+        <v>1192</v>
       </c>
       <c r="D950" s="3" t="inlineStr">
         <is>
-          <t>286372</t>
+          <t>374141</t>
         </is>
       </c>
       <c r="E950" s="3" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>66</t>
         </is>
       </c>
       <c r="F950" s="3" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G950" s="3" t="inlineStr">
         <is>
@@ -30519,24 +30520,24 @@
       </c>
       <c r="B951" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="C951" s="2" t="n">
-        <v>1201</v>
+        <v>1193</v>
       </c>
       <c r="D951" s="2" t="inlineStr">
         <is>
-          <t>284797</t>
+          <t>374310</t>
         </is>
       </c>
       <c r="E951" s="2" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>63</t>
         </is>
       </c>
       <c r="F951" s="2" t="n">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="G951" s="2" t="inlineStr">
         <is>
@@ -30555,20 +30556,20 @@
         </is>
       </c>
       <c r="C952" s="3" t="n">
-        <v>1202</v>
+        <v>1194</v>
       </c>
       <c r="D952" s="3" t="inlineStr">
         <is>
-          <t>284800</t>
+          <t>284796</t>
         </is>
       </c>
       <c r="E952" s="3" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>70</t>
         </is>
       </c>
       <c r="F952" s="3" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G952" s="3" t="inlineStr">
         <is>
@@ -30583,15 +30584,15 @@
       </c>
       <c r="B953" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="C953" s="2" t="n">
-        <v>1203</v>
+        <v>1195</v>
       </c>
       <c r="D953" s="2" t="inlineStr">
         <is>
-          <t>284445</t>
+          <t>286478</t>
         </is>
       </c>
       <c r="E953" s="2" t="inlineStr">
@@ -30600,7 +30601,7 @@
         </is>
       </c>
       <c r="F953" s="2" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G953" s="2" t="inlineStr">
         <is>
@@ -30619,11 +30620,11 @@
         </is>
       </c>
       <c r="C954" s="3" t="n">
-        <v>1205</v>
+        <v>1196</v>
       </c>
       <c r="D954" s="3" t="inlineStr">
         <is>
-          <t>286197</t>
+          <t>286370</t>
         </is>
       </c>
       <c r="E954" s="3" t="inlineStr">
@@ -30632,7 +30633,7 @@
         </is>
       </c>
       <c r="F954" s="3" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="G954" s="3" t="inlineStr">
         <is>
@@ -30647,20 +30648,20 @@
       </c>
       <c r="B955" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="C955" s="2" t="n">
-        <v>1206</v>
+        <v>1197</v>
       </c>
       <c r="D955" s="2" t="inlineStr">
         <is>
-          <t>286401</t>
+          <t>125880</t>
         </is>
       </c>
       <c r="E955" s="2" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>60</t>
         </is>
       </c>
       <c r="F955" s="2" t="n">
@@ -30683,20 +30684,20 @@
         </is>
       </c>
       <c r="C956" s="3" t="n">
-        <v>1209</v>
+        <v>1198</v>
       </c>
       <c r="D956" s="3" t="inlineStr">
         <is>
-          <t>284448</t>
+          <t>286372</t>
         </is>
       </c>
       <c r="E956" s="3" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>74</t>
         </is>
       </c>
       <c r="F956" s="3" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G956" s="3" t="inlineStr">
         <is>
@@ -30711,24 +30712,24 @@
       </c>
       <c r="B957" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="C957" s="2" t="n">
-        <v>1211</v>
+        <v>1199</v>
       </c>
       <c r="D957" s="2" t="inlineStr">
         <is>
-          <t>286198</t>
+          <t>374249</t>
         </is>
       </c>
       <c r="E957" s="2" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>72</t>
         </is>
       </c>
       <c r="F957" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="G957" s="2" t="inlineStr">
         <is>
@@ -30747,20 +30748,20 @@
         </is>
       </c>
       <c r="C958" s="3" t="n">
-        <v>1212</v>
+        <v>1201</v>
       </c>
       <c r="D958" s="3" t="inlineStr">
         <is>
-          <t>284447</t>
+          <t>284797</t>
         </is>
       </c>
       <c r="E958" s="3" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>70</t>
         </is>
       </c>
       <c r="F958" s="3" t="n">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="G958" s="3" t="inlineStr">
         <is>
@@ -30779,27 +30780,539 @@
         </is>
       </c>
       <c r="C959" s="2" t="n">
+        <v>1202</v>
+      </c>
+      <c r="D959" s="2" t="inlineStr">
+        <is>
+          <t>284800</t>
+        </is>
+      </c>
+      <c r="E959" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F959" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="G959" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H959" s="2" t="inlineStr"/>
+    </row>
+    <row r="960" ht="20" customHeight="1">
+      <c r="A960" s="3" t="n">
+        <v>956</v>
+      </c>
+      <c r="B960" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C960" s="3" t="n">
+        <v>1203</v>
+      </c>
+      <c r="D960" s="3" t="inlineStr">
+        <is>
+          <t>284445</t>
+        </is>
+      </c>
+      <c r="E960" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F960" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="G960" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H960" s="3" t="inlineStr"/>
+    </row>
+    <row r="961" ht="20" customHeight="1">
+      <c r="A961" s="2" t="n">
+        <v>957</v>
+      </c>
+      <c r="B961" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C961" s="2" t="n">
+        <v>1205</v>
+      </c>
+      <c r="D961" s="2" t="inlineStr">
+        <is>
+          <t>286197</t>
+        </is>
+      </c>
+      <c r="E961" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F961" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="G961" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H961" s="2" t="inlineStr"/>
+    </row>
+    <row r="962" ht="20" customHeight="1">
+      <c r="A962" s="3" t="n">
+        <v>958</v>
+      </c>
+      <c r="B962" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C962" s="3" t="n">
+        <v>1206</v>
+      </c>
+      <c r="D962" s="3" t="inlineStr">
+        <is>
+          <t>286401</t>
+        </is>
+      </c>
+      <c r="E962" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F962" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="G962" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H962" s="3" t="inlineStr"/>
+    </row>
+    <row r="963" ht="20" customHeight="1">
+      <c r="A963" s="2" t="n">
+        <v>959</v>
+      </c>
+      <c r="B963" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C963" s="2" t="n">
+        <v>1207</v>
+      </c>
+      <c r="D963" s="2" t="inlineStr">
+        <is>
+          <t>125879</t>
+        </is>
+      </c>
+      <c r="E963" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="F963" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="G963" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H963" s="2" t="inlineStr"/>
+    </row>
+    <row r="964" ht="20" customHeight="1">
+      <c r="A964" s="3" t="n">
+        <v>960</v>
+      </c>
+      <c r="B964" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C964" s="3" t="n">
+        <v>1208</v>
+      </c>
+      <c r="D964" s="3" t="inlineStr">
+        <is>
+          <t>374179</t>
+        </is>
+      </c>
+      <c r="E964" s="3" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="F964" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="G964" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H964" s="3" t="inlineStr"/>
+    </row>
+    <row r="965" ht="20" customHeight="1">
+      <c r="A965" s="2" t="n">
+        <v>961</v>
+      </c>
+      <c r="B965" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C965" s="2" t="n">
+        <v>1209</v>
+      </c>
+      <c r="D965" s="2" t="inlineStr">
+        <is>
+          <t>284448</t>
+        </is>
+      </c>
+      <c r="E965" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F965" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G965" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H965" s="2" t="inlineStr"/>
+    </row>
+    <row r="966" ht="20" customHeight="1">
+      <c r="A966" s="3" t="n">
+        <v>962</v>
+      </c>
+      <c r="B966" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C966" s="3" t="n">
+        <v>1211</v>
+      </c>
+      <c r="D966" s="3" t="inlineStr">
+        <is>
+          <t>286198</t>
+        </is>
+      </c>
+      <c r="E966" s="3" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="F966" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="G966" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H966" s="3" t="inlineStr"/>
+    </row>
+    <row r="967" ht="20" customHeight="1">
+      <c r="A967" s="2" t="n">
+        <v>963</v>
+      </c>
+      <c r="B967" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C967" s="2" t="n">
+        <v>1212</v>
+      </c>
+      <c r="D967" s="2" t="inlineStr">
+        <is>
+          <t>284447</t>
+        </is>
+      </c>
+      <c r="E967" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F967" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="G967" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H967" s="2" t="inlineStr"/>
+    </row>
+    <row r="968" ht="20" customHeight="1">
+      <c r="A968" s="3" t="n">
+        <v>964</v>
+      </c>
+      <c r="B968" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C968" s="3" t="n">
+        <v>1213</v>
+      </c>
+      <c r="D968" s="3" t="inlineStr">
+        <is>
+          <t>374143</t>
+        </is>
+      </c>
+      <c r="E968" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F968" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="G968" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H968" s="3" t="inlineStr"/>
+    </row>
+    <row r="969" ht="20" customHeight="1">
+      <c r="A969" s="2" t="n">
+        <v>965</v>
+      </c>
+      <c r="B969" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C969" s="2" t="n">
         <v>1215</v>
       </c>
-      <c r="D959" s="2" t="inlineStr">
+      <c r="D969" s="2" t="inlineStr">
         <is>
           <t>286059</t>
         </is>
       </c>
-      <c r="E959" s="2" t="inlineStr">
+      <c r="E969" s="2" t="inlineStr">
         <is>
           <t>68</t>
         </is>
       </c>
-      <c r="F959" s="2" t="n">
+      <c r="F969" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="G959" s="2" t="inlineStr">
-        <is>
-          <t>SELESAI</t>
-        </is>
-      </c>
-      <c r="H959" s="2" t="inlineStr"/>
+      <c r="G969" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H969" s="2" t="inlineStr"/>
+    </row>
+    <row r="970" ht="20" customHeight="1">
+      <c r="A970" s="3" t="n">
+        <v>966</v>
+      </c>
+      <c r="B970" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C970" s="3" t="n">
+        <v>1216</v>
+      </c>
+      <c r="D970" s="3" t="inlineStr">
+        <is>
+          <t>374142</t>
+        </is>
+      </c>
+      <c r="E970" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F970" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="G970" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H970" s="3" t="inlineStr"/>
+    </row>
+    <row r="971" ht="20" customHeight="1">
+      <c r="A971" s="2" t="n">
+        <v>967</v>
+      </c>
+      <c r="B971" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C971" s="2" t="n">
+        <v>1217</v>
+      </c>
+      <c r="D971" s="2" t="inlineStr">
+        <is>
+          <t>286475</t>
+        </is>
+      </c>
+      <c r="E971" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F971" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="G971" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H971" s="2" t="inlineStr"/>
+    </row>
+    <row r="972" ht="20" customHeight="1">
+      <c r="A972" s="3" t="n">
+        <v>968</v>
+      </c>
+      <c r="B972" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C972" s="3" t="n">
+        <v>1223</v>
+      </c>
+      <c r="D972" s="3" t="inlineStr">
+        <is>
+          <t>374253</t>
+        </is>
+      </c>
+      <c r="E972" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F972" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="G972" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H972" s="3" t="inlineStr"/>
+    </row>
+    <row r="973" ht="20" customHeight="1">
+      <c r="A973" s="2" t="n">
+        <v>969</v>
+      </c>
+      <c r="B973" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C973" s="2" t="n">
+        <v>1224</v>
+      </c>
+      <c r="D973" s="2" t="inlineStr">
+        <is>
+          <t>374251</t>
+        </is>
+      </c>
+      <c r="E973" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F973" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G973" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H973" s="2" t="inlineStr"/>
+    </row>
+    <row r="974" ht="20" customHeight="1">
+      <c r="A974" s="3" t="n">
+        <v>970</v>
+      </c>
+      <c r="B974" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C974" s="3" t="n">
+        <v>1256</v>
+      </c>
+      <c r="D974" s="3" t="inlineStr">
+        <is>
+          <t>374252</t>
+        </is>
+      </c>
+      <c r="E974" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F974" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="G974" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H974" s="3" t="inlineStr"/>
+    </row>
+    <row r="975" ht="20" customHeight="1">
+      <c r="A975" s="2" t="n">
+        <v>971</v>
+      </c>
+      <c r="B975" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C975" s="2" t="n">
+        <v>1261</v>
+      </c>
+      <c r="D975" s="2" t="inlineStr">
+        <is>
+          <t>374666</t>
+        </is>
+      </c>
+      <c r="E975" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F975" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="G975" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H975" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -48489,7 +49002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -48810,6 +49323,501 @@
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>1184</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>374136</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>1189</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>374140</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>1192</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>374141</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>1193</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>374310</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>1195</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>286478</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1197</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>125880</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>1199</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>374249</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>1207</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>125879</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>1208</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>374179</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>1213</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>374143</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>1216</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>374142</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>1217</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>286475</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>1223</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>374253</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>1224</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>374251</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>1256</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>374252</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>No Gudang</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Nomor Barcode</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Berat (Kg)</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>1261</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>374666</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>